<commit_message>
feat(WES Phase B): PB-R3 收尾 — V2 全页面集成 + V0 评估 UX 打磨 + 后端流式支持
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_需求管理/原始需求/需求RR/工作量评估申请表-小鹏汽车集团.xlsx
+++ b/01_需求管理/原始需求/需求RR/工作量评估申请表-小鹏汽车集团.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28260" windowHeight="12320" tabRatio="926" activeTab="1"/>
+    <workbookView windowWidth="24480" windowHeight="16380" tabRatio="926" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="填写说明" sheetId="2" r:id="rId1"/>
@@ -357,7 +357,7 @@
     <t>企业简介</t>
   </si>
   <si>
-    <t xml:space="preserve">广东小鹏汽车集团有限公司，整车制造行业企业，2025年营收767.2亿元。本次项目涉及集团及子公司共2家组织，实施地点位于东莞，主营整车制造业务，需建设数字化ERP平台支撑业务发展。 </t>
+    <t xml:space="preserve">广东小鹏汽车集团有限公司，整车制造行业企业，2025年营收767.2亿元。本次项目涉及集团及子公司共2家组织，实施地点位于广州黄埔，主营整车制造业务，需建设数字化ERP平台支撑业务发展。 </t>
   </si>
   <si>
     <t>项目背景和需求</t>
@@ -1518,6 +1518,17 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="thin">
+        <color theme="0" tint="-0.499984740745262"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.499984740745262"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color theme="0" tint="-0.499984740745262"/>
       </left>
@@ -1535,17 +1546,6 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="0" tint="-0.499984740745262"/>
-      </right>
-      <top style="thin">
-        <color theme="0" tint="-0.499984740745262"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -2005,6 +2005,9 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2015,9 +2018,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2042,6 +2042,9 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -2057,9 +2060,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2072,20 +2072,20 @@
     <xf numFmtId="0" fontId="15" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="52" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2103,25 +2103,25 @@
     <xf numFmtId="0" fontId="17" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3091,15 +3091,15 @@
     <col min="3" max="16384" width="8.66071428571429" style="82"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30.5" customHeight="1" spans="2:2">
+    <row r="1" ht="30.5" customHeight="1" spans="2:6">
       <c r="B1" s="83" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" ht="14.25" customHeight="1" spans="2:2">
+    <row r="2" ht="14.25" customHeight="1" spans="2:6">
       <c r="B2" s="84"/>
     </row>
-    <row r="3" ht="14.25" customHeight="1" spans="2:2">
+    <row r="3" ht="14.25" customHeight="1" spans="2:6">
       <c r="B3" s="84"/>
     </row>
     <row r="9" ht="19.5" customHeight="1"/>
@@ -3124,76 +3124,76 @@
       <c r="E12" s="85"/>
       <c r="F12" s="85"/>
     </row>
-    <row r="13" spans="2:5">
+    <row r="13" spans="2:6">
       <c r="B13" s="90" t="s">
         <v>4</v>
       </c>
       <c r="E13" s="85"/>
     </row>
-    <row r="14" spans="2:5">
+    <row r="14" spans="2:6">
       <c r="B14" s="90" t="s">
         <v>5</v>
       </c>
       <c r="E14" s="85"/>
     </row>
-    <row r="15" spans="2:5">
+    <row r="15" spans="2:6">
       <c r="B15" s="90" t="s">
         <v>6</v>
       </c>
       <c r="E15" s="85"/>
     </row>
-    <row r="16" spans="2:5">
+    <row r="16" spans="2:6">
       <c r="B16" s="90" t="s">
         <v>7</v>
       </c>
       <c r="E16" s="85"/>
     </row>
-    <row r="17" spans="2:5">
+    <row r="17" spans="2:13">
       <c r="B17" s="90" t="s">
         <v>8</v>
       </c>
       <c r="E17" s="85"/>
     </row>
-    <row r="18" spans="2:5">
+    <row r="18" spans="2:13">
       <c r="B18" s="85"/>
       <c r="E18" s="85"/>
     </row>
-    <row r="19" ht="27" customHeight="1" spans="2:4">
+    <row r="19" ht="27" customHeight="1" spans="2:13">
       <c r="B19" s="83" t="s">
         <v>9</v>
       </c>
       <c r="C19" s="86"/>
       <c r="D19" s="86"/>
     </row>
-    <row r="20" ht="16.5" customHeight="1" spans="2:4">
+    <row r="20" ht="16.5" customHeight="1" spans="2:13">
       <c r="B20" s="84" t="s">
         <v>10</v>
       </c>
       <c r="C20" s="86"/>
       <c r="D20" s="86"/>
     </row>
-    <row r="21" spans="2:4">
+    <row r="21" spans="2:13">
       <c r="B21" s="91" t="s">
         <v>11</v>
       </c>
       <c r="C21" s="86"/>
       <c r="D21" s="86"/>
     </row>
-    <row r="22" spans="2:4">
+    <row r="22" spans="2:13">
       <c r="B22" s="91" t="s">
         <v>12</v>
       </c>
       <c r="C22" s="86"/>
       <c r="D22" s="86"/>
     </row>
-    <row r="23" spans="2:4">
+    <row r="23" spans="2:13">
       <c r="B23" s="91" t="s">
         <v>13</v>
       </c>
       <c r="C23" s="86"/>
       <c r="D23" s="86"/>
     </row>
-    <row r="24" ht="17.6" spans="2:4">
+    <row r="24" ht="17.6" spans="2:13">
       <c r="B24" s="84" t="s">
         <v>14</v>
       </c>
@@ -3248,27 +3248,27 @@
       <c r="L27" s="89"/>
       <c r="M27" s="89"/>
     </row>
-    <row r="28" spans="2:4">
+    <row r="28" spans="2:13">
       <c r="B28" s="87"/>
       <c r="C28" s="86"/>
       <c r="D28" s="86"/>
     </row>
-    <row r="29" spans="2:4">
+    <row r="29" spans="2:13">
       <c r="B29" s="87"/>
       <c r="C29" s="86"/>
       <c r="D29" s="86"/>
     </row>
-    <row r="30" spans="2:4">
+    <row r="30" spans="2:13">
       <c r="B30" s="87"/>
       <c r="C30" s="86"/>
       <c r="D30" s="86"/>
     </row>
-    <row r="31" ht="17.6" spans="2:4">
+    <row r="31" ht="17.6" spans="2:13">
       <c r="B31" s="84"/>
       <c r="C31" s="86"/>
       <c r="D31" s="86"/>
     </row>
-    <row r="32" spans="2:4">
+    <row r="32" spans="2:13">
       <c r="B32" s="87"/>
       <c r="C32" s="86"/>
       <c r="D32" s="86"/>
@@ -3278,10 +3278,10 @@
       <c r="C33" s="86"/>
       <c r="D33" s="86"/>
     </row>
-    <row r="34" spans="2:2">
+    <row r="34" spans="2:4">
       <c r="B34" s="88"/>
     </row>
-    <row r="35" spans="2:2">
+    <row r="35" spans="2:4">
       <c r="B35" s="88"/>
     </row>
   </sheetData>
@@ -3804,7 +3804,7 @@
     <col min="16133" max="16384" width="8.16071428571429" style="61"/>
   </cols>
   <sheetData>
-    <row r="1" ht="29.5" customHeight="1" spans="1:4">
+    <row r="1" ht="29.5" customHeight="1" spans="1:9">
       <c r="A1" s="62" t="s">
         <v>37</v>
       </c>
@@ -3812,7 +3812,7 @@
       <c r="C1" s="62"/>
       <c r="D1" s="62"/>
     </row>
-    <row r="2" s="60" customFormat="1" spans="1:4">
+    <row r="2" s="60" customFormat="1" spans="1:9">
       <c r="A2" s="63" t="s">
         <v>38</v>
       </c>
@@ -3826,7 +3826,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" ht="46" spans="1:6">
+    <row r="3" ht="46" spans="1:9">
       <c r="A3" s="65" t="s">
         <v>42</v>
       </c>
@@ -3838,7 +3838,7 @@
       <c r="E3" s="68"/>
       <c r="F3" s="68"/>
     </row>
-    <row r="4" ht="16.8" spans="2:9">
+    <row r="4" ht="16.8" spans="1:9">
       <c r="B4"/>
       <c r="C4"/>
       <c r="D4"/>
@@ -3848,7 +3848,7 @@
       <c r="H4"/>
       <c r="I4"/>
     </row>
-    <row r="5" ht="16.8" spans="2:9">
+    <row r="5" ht="16.8" spans="1:9">
       <c r="B5"/>
       <c r="C5"/>
       <c r="D5"/>
@@ -3858,7 +3858,7 @@
       <c r="H5"/>
       <c r="I5"/>
     </row>
-    <row r="6" ht="16.8" spans="2:9">
+    <row r="6" ht="16.8" spans="1:9">
       <c r="B6"/>
       <c r="C6"/>
       <c r="D6"/>
@@ -3868,7 +3868,7 @@
       <c r="H6"/>
       <c r="I6"/>
     </row>
-    <row r="7" ht="16.8" spans="2:9">
+    <row r="7" ht="16.8" spans="1:9">
       <c r="B7"/>
       <c r="C7"/>
       <c r="D7"/>
@@ -3878,7 +3878,7 @@
       <c r="H7"/>
       <c r="I7"/>
     </row>
-    <row r="8" ht="16.8" spans="2:9">
+    <row r="8" ht="16.8" spans="1:9">
       <c r="B8"/>
       <c r="C8"/>
       <c r="D8"/>
@@ -3888,7 +3888,7 @@
       <c r="H8"/>
       <c r="I8"/>
     </row>
-    <row r="9" ht="16.8" spans="2:9">
+    <row r="9" ht="16.8" spans="1:9">
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9"/>
@@ -3898,7 +3898,7 @@
       <c r="H9"/>
       <c r="I9"/>
     </row>
-    <row r="10" ht="16.8" spans="2:9">
+    <row r="10" ht="16.8" spans="1:9">
       <c r="B10"/>
       <c r="C10"/>
       <c r="D10"/>
@@ -3908,7 +3908,7 @@
       <c r="H10"/>
       <c r="I10"/>
     </row>
-    <row r="11" ht="16.8" spans="2:9">
+    <row r="11" ht="16.8" spans="1:9">
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11"/>
@@ -3918,7 +3918,7 @@
       <c r="H11"/>
       <c r="I11"/>
     </row>
-    <row r="12" ht="16.8" spans="2:9">
+    <row r="12" ht="16.8" spans="1:9">
       <c r="B12"/>
       <c r="C12"/>
       <c r="D12"/>
@@ -3928,7 +3928,7 @@
       <c r="H12"/>
       <c r="I12"/>
     </row>
-    <row r="13" ht="16.8" spans="2:9">
+    <row r="13" ht="16.8" spans="1:9">
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13"/>
@@ -3938,7 +3938,7 @@
       <c r="H13"/>
       <c r="I13"/>
     </row>
-    <row r="14" ht="16.8" spans="2:9">
+    <row r="14" ht="16.8" spans="1:9">
       <c r="B14"/>
       <c r="C14"/>
       <c r="D14"/>
@@ -3948,7 +3948,7 @@
       <c r="H14"/>
       <c r="I14"/>
     </row>
-    <row r="15" ht="16.8" spans="2:9">
+    <row r="15" ht="16.8" spans="1:9">
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15"/>
@@ -3958,7 +3958,7 @@
       <c r="H15"/>
       <c r="I15"/>
     </row>
-    <row r="16" ht="16.8" spans="2:9">
+    <row r="16" ht="16.8" spans="1:9">
       <c r="B16"/>
       <c r="C16"/>
       <c r="D16"/>
@@ -4275,19 +4275,19 @@
       <c r="G1" s="53"/>
       <c r="H1" s="53"/>
       <c r="I1" s="53"/>
-      <c r="J1" s="58"/>
+      <c r="J1" s="54"/>
     </row>
     <row r="2" ht="14" customHeight="1" spans="1:10">
-      <c r="A2" s="54"/>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="59"/>
+      <c r="A2" s="55"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="57"/>
     </row>
     <row r="3" ht="18.5" customHeight="1" spans="1:10">
       <c r="A3" s="44" t="s">
@@ -4322,162 +4322,162 @@
       </c>
     </row>
     <row r="4" ht="45" customHeight="1" spans="1:10">
-      <c r="A4" s="56">
+      <c r="A4" s="58">
         <v>1</v>
       </c>
-      <c r="B4" s="56" t="s">
+      <c r="B4" s="58" t="s">
         <v>54</v>
       </c>
-      <c r="C4" s="56" t="s">
+      <c r="C4" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="D4" s="57" t="s">
+      <c r="D4" s="59" t="s">
         <v>56</v>
       </c>
-      <c r="E4" s="56" t="s">
+      <c r="E4" s="58" t="s">
         <v>57</v>
       </c>
-      <c r="F4" s="56" t="s">
+      <c r="F4" s="58" t="s">
         <v>58</v>
       </c>
-      <c r="G4" s="56" t="s">
+      <c r="G4" s="58" t="s">
         <v>59</v>
       </c>
-      <c r="H4" s="56" t="s">
+      <c r="H4" s="58" t="s">
         <v>60</v>
       </c>
-      <c r="I4" s="57" t="s">
+      <c r="I4" s="59" t="s">
         <v>61</v>
       </c>
-      <c r="J4" s="56" t="s">
+      <c r="J4" s="58" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:10">
-      <c r="A5" s="56">
+      <c r="A5" s="58">
         <v>2</v>
       </c>
-      <c r="B5" s="56" t="s">
+      <c r="B5" s="58" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="56" t="s">
+      <c r="C5" s="58" t="s">
         <v>63</v>
       </c>
-      <c r="D5" s="57" t="s">
+      <c r="D5" s="59" t="s">
         <v>64</v>
       </c>
-      <c r="E5" s="56" t="s">
+      <c r="E5" s="58" t="s">
         <v>57</v>
       </c>
-      <c r="F5" s="56" t="s">
+      <c r="F5" s="58" t="s">
         <v>58</v>
       </c>
-      <c r="G5" s="56" t="s">
+      <c r="G5" s="58" t="s">
         <v>59</v>
       </c>
-      <c r="H5" s="56" t="s">
+      <c r="H5" s="58" t="s">
         <v>60</v>
       </c>
-      <c r="I5" s="57" t="s">
+      <c r="I5" s="59" t="s">
         <v>65</v>
       </c>
-      <c r="J5" s="56" t="s">
+      <c r="J5" s="58" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:10">
-      <c r="A6" s="56">
+      <c r="A6" s="58">
         <v>3</v>
       </c>
-      <c r="B6" s="56" t="s">
+      <c r="B6" s="58" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="56" t="s">
+      <c r="C6" s="58" t="s">
         <v>66</v>
       </c>
-      <c r="D6" s="57" t="s">
+      <c r="D6" s="59" t="s">
         <v>67</v>
       </c>
-      <c r="E6" s="56" t="s">
+      <c r="E6" s="58" t="s">
         <v>57</v>
       </c>
-      <c r="F6" s="56" t="s">
+      <c r="F6" s="58" t="s">
         <v>58</v>
       </c>
-      <c r="G6" s="56" t="s">
+      <c r="G6" s="58" t="s">
         <v>59</v>
       </c>
-      <c r="H6" s="56" t="s">
+      <c r="H6" s="58" t="s">
         <v>60</v>
       </c>
-      <c r="I6" s="57" t="s">
+      <c r="I6" s="59" t="s">
         <v>68</v>
       </c>
-      <c r="J6" s="56" t="s">
+      <c r="J6" s="58" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:10">
-      <c r="A7" s="56">
+      <c r="A7" s="58">
         <v>4</v>
       </c>
-      <c r="B7" s="56" t="s">
+      <c r="B7" s="58" t="s">
         <v>69</v>
       </c>
-      <c r="C7" s="56" t="s">
+      <c r="C7" s="58" t="s">
         <v>69</v>
       </c>
-      <c r="D7" s="47" t="s">
+      <c r="D7" s="48" t="s">
         <v>70</v>
       </c>
-      <c r="E7" s="56" t="s">
+      <c r="E7" s="58" t="s">
         <v>57</v>
       </c>
-      <c r="F7" s="56" t="s">
+      <c r="F7" s="58" t="s">
         <v>58</v>
       </c>
-      <c r="G7" s="56" t="s">
+      <c r="G7" s="58" t="s">
         <v>59</v>
       </c>
-      <c r="H7" s="56" t="s">
+      <c r="H7" s="58" t="s">
         <v>60</v>
       </c>
-      <c r="I7" s="57" t="s">
+      <c r="I7" s="59" t="s">
         <v>71</v>
       </c>
-      <c r="J7" s="56" t="s">
+      <c r="J7" s="58" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="8" ht="65" customHeight="1" spans="1:10">
-      <c r="A8" s="56">
+      <c r="A8" s="58">
         <v>5</v>
       </c>
-      <c r="B8" s="56" t="s">
+      <c r="B8" s="58" t="s">
         <v>72</v>
       </c>
-      <c r="C8" s="56" t="s">
+      <c r="C8" s="58" t="s">
         <v>73</v>
       </c>
-      <c r="D8" s="47" t="s">
+      <c r="D8" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="E8" s="56" t="s">
+      <c r="E8" s="58" t="s">
         <v>57</v>
       </c>
-      <c r="F8" s="56" t="s">
+      <c r="F8" s="58" t="s">
         <v>58</v>
       </c>
-      <c r="G8" s="56" t="s">
+      <c r="G8" s="58" t="s">
         <v>59</v>
       </c>
-      <c r="H8" s="56" t="s">
+      <c r="H8" s="58" t="s">
         <v>75</v>
       </c>
-      <c r="I8" s="57" t="s">
+      <c r="I8" s="59" t="s">
         <v>76</v>
       </c>
-      <c r="J8" s="56" t="s">
+      <c r="J8" s="58" t="s">
         <v>77</v>
       </c>
     </row>
@@ -4535,7 +4535,7 @@
       <c r="I1" s="44" t="s">
         <v>84</v>
       </c>
-      <c r="J1" s="50" t="s">
+      <c r="J1" s="46" t="s">
         <v>85</v>
       </c>
     </row>
@@ -4543,16 +4543,16 @@
       <c r="A2" s="31" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="47" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="46" t="s">
+      <c r="C2" s="47" t="s">
         <v>55</v>
       </c>
-      <c r="D2" s="47" t="s">
+      <c r="D2" s="48" t="s">
         <v>86</v>
       </c>
-      <c r="E2" s="27" t="s">
+      <c r="E2" s="28" t="s">
         <v>87</v>
       </c>
       <c r="F2" s="49">
@@ -4570,7 +4570,7 @@
         <f>SUM(F2:H2)</f>
         <v>2.4</v>
       </c>
-      <c r="J2" s="27" t="s">
+      <c r="J2" s="28" t="s">
         <v>88</v>
       </c>
     </row>
@@ -4578,16 +4578,16 @@
       <c r="A3" s="31" t="s">
         <v>54</v>
       </c>
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="47" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="46" t="s">
+      <c r="C3" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="D3" s="47" t="s">
+      <c r="D3" s="48" t="s">
         <v>89</v>
       </c>
-      <c r="E3" s="27" t="s">
+      <c r="E3" s="28" t="s">
         <v>87</v>
       </c>
       <c r="F3" s="49">
@@ -4605,22 +4605,22 @@
         <f>SUM(F3:H3)</f>
         <v>2.4</v>
       </c>
-      <c r="J3" s="27"/>
+      <c r="J3" s="28"/>
     </row>
     <row r="4" ht="27" customHeight="1" spans="1:10">
       <c r="A4" s="31" t="s">
         <v>54</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="47" t="s">
         <v>54</v>
       </c>
-      <c r="C4" s="46" t="s">
+      <c r="C4" s="47" t="s">
         <v>66</v>
       </c>
-      <c r="D4" s="47" t="s">
+      <c r="D4" s="48" t="s">
         <v>90</v>
       </c>
-      <c r="E4" s="27" t="s">
+      <c r="E4" s="28" t="s">
         <v>87</v>
       </c>
       <c r="F4" s="49">
@@ -4638,7 +4638,7 @@
         <f>SUM(F4:H4)</f>
         <v>4.8</v>
       </c>
-      <c r="J4" s="27"/>
+      <c r="J4" s="28"/>
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:10">
       <c r="A5" s="31" t="s">
@@ -4647,13 +4647,13 @@
       <c r="B5" s="31" t="s">
         <v>91</v>
       </c>
-      <c r="C5" s="46" t="s">
+      <c r="C5" s="47" t="s">
         <v>92</v>
       </c>
-      <c r="D5" s="47" t="s">
+      <c r="D5" s="48" t="s">
         <v>93</v>
       </c>
-      <c r="E5" s="27" t="s">
+      <c r="E5" s="28" t="s">
         <v>87</v>
       </c>
       <c r="F5" s="49">
@@ -4671,7 +4671,7 @@
         <f>SUM(F5:H5)</f>
         <v>2.4</v>
       </c>
-      <c r="J5" s="27"/>
+      <c r="J5" s="28"/>
     </row>
     <row r="6" ht="28" customHeight="1" spans="1:10">
       <c r="A6" s="31" t="s">
@@ -4680,13 +4680,13 @@
       <c r="B6" s="31" t="s">
         <v>91</v>
       </c>
-      <c r="C6" s="46" t="s">
+      <c r="C6" s="47" t="s">
         <v>94</v>
       </c>
-      <c r="D6" s="47" t="s">
+      <c r="D6" s="48" t="s">
         <v>95</v>
       </c>
-      <c r="E6" s="27" t="s">
+      <c r="E6" s="28" t="s">
         <v>87</v>
       </c>
       <c r="F6" s="49">
@@ -4704,20 +4704,20 @@
         <f>SUM(F6:H6)</f>
         <v>4.8</v>
       </c>
-      <c r="J6" s="27"/>
+      <c r="J6" s="28"/>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:10">
-      <c r="A7" s="48" t="s">
+      <c r="A7" s="50" t="s">
         <v>96</v>
       </c>
-      <c r="B7" s="48"/>
-      <c r="C7" s="48"/>
-      <c r="D7" s="48"/>
-      <c r="E7" s="48"/>
-      <c r="F7" s="46"/>
-      <c r="G7" s="46"/>
-      <c r="H7" s="46"/>
-      <c r="I7" s="28">
+      <c r="B7" s="50"/>
+      <c r="C7" s="50"/>
+      <c r="D7" s="50"/>
+      <c r="E7" s="50"/>
+      <c r="F7" s="47"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="47"/>
+      <c r="I7" s="29">
         <f>SUM(I2:I6)</f>
         <v>16.8</v>
       </c>
@@ -4788,16 +4788,16 @@
       <c r="D2" s="36">
         <v>10</v>
       </c>
-      <c r="E2" s="41">
+      <c r="E2" s="37">
         <v>2</v>
       </c>
-      <c r="F2" s="41" t="s">
+      <c r="F2" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="G2" s="41">
+      <c r="G2" s="37">
         <v>2</v>
       </c>
-      <c r="H2" s="41" t="s">
+      <c r="H2" s="37" t="s">
         <v>108</v>
       </c>
     </row>
@@ -4808,16 +4808,16 @@
         <v>109</v>
       </c>
       <c r="D3" s="36"/>
-      <c r="E3" s="41">
+      <c r="E3" s="37">
         <v>2</v>
       </c>
-      <c r="F3" s="41" t="s">
+      <c r="F3" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="G3" s="41">
+      <c r="G3" s="37">
         <v>2</v>
       </c>
-      <c r="H3" s="41" t="s">
+      <c r="H3" s="37" t="s">
         <v>108</v>
       </c>
     </row>
@@ -4828,16 +4828,16 @@
         <v>110</v>
       </c>
       <c r="D4" s="36"/>
-      <c r="E4" s="41">
+      <c r="E4" s="37">
         <v>2</v>
       </c>
-      <c r="F4" s="41" t="s">
+      <c r="F4" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="G4" s="41">
+      <c r="G4" s="37">
         <v>2</v>
       </c>
-      <c r="H4" s="41" t="s">
+      <c r="H4" s="37" t="s">
         <v>108</v>
       </c>
     </row>
@@ -4848,16 +4848,16 @@
         <v>111</v>
       </c>
       <c r="D5" s="36"/>
-      <c r="E5" s="41">
+      <c r="E5" s="37">
         <v>2</v>
       </c>
-      <c r="F5" s="41" t="s">
+      <c r="F5" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="G5" s="41">
+      <c r="G5" s="37">
         <v>2</v>
       </c>
-      <c r="H5" s="41" t="s">
+      <c r="H5" s="37" t="s">
         <v>108</v>
       </c>
     </row>
@@ -4868,16 +4868,16 @@
         <v>112</v>
       </c>
       <c r="D6" s="36"/>
-      <c r="E6" s="41">
+      <c r="E6" s="37">
         <v>2</v>
       </c>
-      <c r="F6" s="41" t="s">
+      <c r="F6" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="G6" s="41">
+      <c r="G6" s="37">
         <v>2</v>
       </c>
-      <c r="H6" s="41" t="s">
+      <c r="H6" s="37" t="s">
         <v>108</v>
       </c>
     </row>
@@ -4888,16 +4888,16 @@
         <v>113</v>
       </c>
       <c r="D7" s="36"/>
-      <c r="E7" s="41">
+      <c r="E7" s="37">
         <v>2</v>
       </c>
-      <c r="F7" s="41" t="s">
+      <c r="F7" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="G7" s="41">
+      <c r="G7" s="37">
         <v>2</v>
       </c>
-      <c r="H7" s="41" t="s">
+      <c r="H7" s="37" t="s">
         <v>108</v>
       </c>
     </row>
@@ -4908,16 +4908,16 @@
         <v>114</v>
       </c>
       <c r="D8" s="36"/>
-      <c r="E8" s="41">
+      <c r="E8" s="37">
         <v>2</v>
       </c>
-      <c r="F8" s="41" t="s">
+      <c r="F8" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="G8" s="41">
+      <c r="G8" s="37">
         <v>2</v>
       </c>
-      <c r="H8" s="41" t="s">
+      <c r="H8" s="37" t="s">
         <v>108</v>
       </c>
     </row>
@@ -4928,16 +4928,16 @@
         <v>115</v>
       </c>
       <c r="D9" s="36"/>
-      <c r="E9" s="41">
+      <c r="E9" s="37">
         <v>2</v>
       </c>
-      <c r="F9" s="41" t="s">
+      <c r="F9" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="G9" s="41">
+      <c r="G9" s="37">
         <v>2</v>
       </c>
-      <c r="H9" s="41" t="s">
+      <c r="H9" s="37" t="s">
         <v>108</v>
       </c>
     </row>
@@ -4948,120 +4948,120 @@
         <v>116</v>
       </c>
       <c r="D10" s="36"/>
-      <c r="E10" s="41">
+      <c r="E10" s="37">
         <v>2</v>
       </c>
-      <c r="F10" s="41" t="s">
+      <c r="F10" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="G10" s="41">
+      <c r="G10" s="37">
         <v>2</v>
       </c>
-      <c r="H10" s="41" t="s">
+      <c r="H10" s="37" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="11" customHeight="1" spans="1:8">
       <c r="A11" s="33"/>
-      <c r="B11" s="37" t="s">
+      <c r="B11" s="38" t="s">
         <v>117</v>
       </c>
       <c r="C11" s="35" t="s">
         <v>118</v>
       </c>
       <c r="D11" s="36"/>
-      <c r="E11" s="41">
+      <c r="E11" s="37">
         <v>2</v>
       </c>
-      <c r="F11" s="41" t="s">
+      <c r="F11" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="G11" s="41">
+      <c r="G11" s="37">
         <v>2</v>
       </c>
-      <c r="H11" s="41" t="s">
+      <c r="H11" s="37" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="12" customHeight="1" spans="1:8">
       <c r="A12" s="33"/>
-      <c r="B12" s="38"/>
+      <c r="B12" s="39"/>
       <c r="C12" s="35" t="s">
         <v>119</v>
       </c>
       <c r="D12" s="36"/>
-      <c r="E12" s="41">
+      <c r="E12" s="37">
         <v>2</v>
       </c>
-      <c r="F12" s="41" t="s">
+      <c r="F12" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="G12" s="41">
+      <c r="G12" s="37">
         <v>2</v>
       </c>
-      <c r="H12" s="41" t="s">
+      <c r="H12" s="37" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="13" customHeight="1" spans="1:8">
       <c r="A13" s="33"/>
-      <c r="B13" s="38"/>
+      <c r="B13" s="39"/>
       <c r="C13" s="35" t="s">
         <v>120</v>
       </c>
       <c r="D13" s="36"/>
-      <c r="E13" s="41">
+      <c r="E13" s="37">
         <v>2</v>
       </c>
-      <c r="F13" s="41" t="s">
+      <c r="F13" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="G13" s="41">
+      <c r="G13" s="37">
         <v>2</v>
       </c>
-      <c r="H13" s="41" t="s">
+      <c r="H13" s="37" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="14" customHeight="1" spans="1:8">
       <c r="A14" s="33"/>
-      <c r="B14" s="39"/>
+      <c r="B14" s="40"/>
       <c r="C14" s="35" t="s">
         <v>121</v>
       </c>
       <c r="D14" s="36"/>
-      <c r="E14" s="41">
+      <c r="E14" s="37">
         <v>2</v>
       </c>
-      <c r="F14" s="41" t="s">
+      <c r="F14" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="G14" s="41">
+      <c r="G14" s="37">
         <v>2</v>
       </c>
-      <c r="H14" s="41" t="s">
+      <c r="H14" s="37" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="15" customHeight="1" spans="1:8">
       <c r="A15" s="33"/>
-      <c r="B15" s="39" t="s">
+      <c r="B15" s="40" t="s">
         <v>122</v>
       </c>
       <c r="C15" s="35" t="s">
         <v>123</v>
       </c>
       <c r="D15" s="36"/>
-      <c r="E15" s="41">
+      <c r="E15" s="37">
         <v>2</v>
       </c>
-      <c r="F15" s="41" t="s">
+      <c r="F15" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="G15" s="41">
+      <c r="G15" s="37">
         <v>2</v>
       </c>
-      <c r="H15" s="41" t="s">
+      <c r="H15" s="37" t="s">
         <v>108</v>
       </c>
     </row>
@@ -5070,22 +5070,22 @@
       <c r="B16" s="34" t="s">
         <v>124</v>
       </c>
-      <c r="C16" s="40" t="s">
+      <c r="C16" s="41" t="s">
         <v>125</v>
       </c>
-      <c r="D16" s="41">
+      <c r="D16" s="37">
         <v>50</v>
       </c>
-      <c r="E16" s="41">
+      <c r="E16" s="37">
         <v>2</v>
       </c>
-      <c r="F16" s="41" t="s">
+      <c r="F16" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="G16" s="41">
+      <c r="G16" s="37">
         <v>2</v>
       </c>
-      <c r="H16" s="41" t="s">
+      <c r="H16" s="37" t="s">
         <v>108</v>
       </c>
     </row>
@@ -5133,27 +5133,27 @@
       <c r="E1" s="24" t="s">
         <v>129</v>
       </c>
-      <c r="F1" s="29" t="s">
+      <c r="F1" s="25" t="s">
         <v>130</v>
       </c>
-      <c r="G1" s="29" t="s">
+      <c r="G1" s="25" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:7">
-      <c r="A2" s="25">
+      <c r="A2" s="26">
         <v>1</v>
       </c>
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C2" s="28" t="s">
         <v>132</v>
       </c>
-      <c r="D2" s="28" t="s">
+      <c r="D2" s="29" t="s">
         <v>133</v>
       </c>
-      <c r="E2" s="28" t="s">
+      <c r="E2" s="29" t="s">
         <v>134</v>
       </c>
       <c r="F2" s="30" t="s">
@@ -5162,19 +5162,19 @@
       <c r="G2" s="31"/>
     </row>
     <row r="3" ht="33" customHeight="1" spans="1:7">
-      <c r="A3" s="25">
+      <c r="A3" s="26">
         <v>2</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="27" t="s">
         <v>136</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="C3" s="28" t="s">
         <v>132</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="29" t="s">
         <v>133</v>
       </c>
-      <c r="E3" s="28" t="s">
+      <c r="E3" s="29" t="s">
         <v>134</v>
       </c>
       <c r="F3" s="30" t="s">

</xml_diff>